<commit_message>
Fix unit_cost_interpolation to apply six-tenths CAPEX scaling
Branch on the dict key, not the numeric value: 'CAPEX' in k -> r**0.6,
'OPEX' in k -> r**0.7, else linear. Previously the isinstance(v, str)
guard sent every numeric cost to the linear branch, making the
six-tenths and OPEX-0.7 rules dead code (CCS/PSA/R-510 scaled linearly).

Post-fix: CCS MJSP premium shrinks with scale (0.207->0.139) and CCS
abatement falls with scale (251->168 $/t alloc) instead of staying flat.
Base-scale CCS/PSA/R-510 costs rise, so base MJSP de-syncs from the
manuscript (generated under the linear bug). Report updated (section 4).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016MjFwwDgUpjrZDZMd1ma7x
</commit_message>
<xml_diff>
--- a/Result/ScaleUp_Sensitivity_table.xlsx
+++ b/Result/ScaleUp_Sensitivity_table.xlsx
@@ -503,31 +503,31 @@
         <v>0.0486490000024665</v>
       </c>
       <c r="D2" t="n">
-        <v>428664382.2549371</v>
+        <v>450905639.8717471</v>
       </c>
       <c r="E2" t="n">
-        <v>133352061.7145777</v>
+        <v>133337434.4285637</v>
       </c>
       <c r="F2" t="n">
-        <v>1.581820719277321</v>
+        <v>1.638403452772569</v>
       </c>
       <c r="G2" t="n">
-        <v>501268882.2549371</v>
+        <v>523510139.8717471</v>
       </c>
       <c r="H2" t="n">
-        <v>230000132.6105777</v>
+        <v>229985505.3245637</v>
       </c>
       <c r="I2" t="n">
-        <v>3.425950976640018</v>
+        <v>3.482533710135268</v>
       </c>
       <c r="J2" t="n">
-        <v>446451718.8964491</v>
+        <v>486640005.7415572</v>
       </c>
       <c r="K2" t="n">
-        <v>139907615.1180534</v>
+        <v>139892987.8320395</v>
       </c>
       <c r="L2" t="n">
-        <v>1.742620522667315</v>
+        <v>1.845068955589855</v>
       </c>
     </row>
     <row r="3">
@@ -541,31 +541,31 @@
         <v>0.0486490000002637</v>
       </c>
       <c r="D3" t="n">
-        <v>888237455.6460499</v>
+        <v>915251977.8238976</v>
       </c>
       <c r="E3" t="n">
-        <v>310142504.2576723</v>
+        <v>310094448.2498837</v>
       </c>
       <c r="F3" t="n">
-        <v>1.230774069524986</v>
+        <v>1.258051347814137</v>
       </c>
       <c r="G3" t="n">
-        <v>1027445455.64605</v>
+        <v>1054459977.823898</v>
       </c>
       <c r="H3" t="n">
-        <v>548996251.2816722</v>
+        <v>548948195.2738836</v>
       </c>
       <c r="I3" t="n">
-        <v>3.022162605305231</v>
+        <v>3.049439883594382</v>
       </c>
       <c r="J3" t="n">
-        <v>932705796.9377314</v>
+        <v>977174706.1283325</v>
       </c>
       <c r="K3" t="n">
-        <v>326531388.1418637</v>
+        <v>326483332.1340751</v>
       </c>
       <c r="L3" t="n">
-        <v>1.391573873960496</v>
+        <v>1.436693830318925</v>
       </c>
     </row>
     <row r="4">
@@ -579,31 +579,31 @@
         <v>0.04864899999956315</v>
       </c>
       <c r="D4" t="n">
-        <v>1653526911.2921</v>
+        <v>1676281957.945513</v>
       </c>
       <c r="E4" t="n">
-        <v>573602208.5153446</v>
+        <v>573492462.3222957</v>
       </c>
       <c r="F4" t="n">
-        <v>1.003659653005043</v>
+        <v>1.014904093554843</v>
       </c>
       <c r="G4" t="n">
-        <v>1908785911.2921</v>
+        <v>1931540957.945513</v>
       </c>
       <c r="H4" t="n">
-        <v>1049772885.763345</v>
+        <v>1049663139.570296</v>
       </c>
       <c r="I4" t="n">
-        <v>2.777804183411691</v>
+        <v>2.789048623961491</v>
       </c>
       <c r="J4" t="n">
-        <v>1742463593.875463</v>
+        <v>1770139263.080067</v>
       </c>
       <c r="K4" t="n">
-        <v>606379976.2811972</v>
+        <v>606270230.0881482</v>
       </c>
       <c r="L4" t="n">
-        <v>1.164459457431652</v>
+        <v>1.178218941449239</v>
       </c>
     </row>
     <row r="5">
@@ -617,31 +617,31 @@
         <v>0.04864899999932714</v>
       </c>
       <c r="D5" t="n">
-        <v>2338195379.843129</v>
+        <v>2350346095.831089</v>
       </c>
       <c r="E5" t="n">
-        <v>828523312.8822664</v>
+        <v>828348559.9508667</v>
       </c>
       <c r="F5" t="n">
-        <v>0.880452523587846</v>
+        <v>0.8841829024748166</v>
       </c>
       <c r="G5" t="n">
-        <v>2710883379.843129</v>
+        <v>2723034095.831089</v>
       </c>
       <c r="H5" t="n">
-        <v>1540147963.954266</v>
+        <v>1539973211.022866</v>
       </c>
       <c r="I5" t="n">
-        <v>2.644947764705025</v>
+        <v>2.648678143591995</v>
       </c>
       <c r="J5" t="n">
-        <v>2471600404.908844</v>
+        <v>2470054003.003464</v>
       </c>
       <c r="K5" t="n">
-        <v>877689903.6907455</v>
+        <v>877515150.7593458</v>
       </c>
       <c r="L5" t="n">
-        <v>1.041252144908923</v>
+        <v>1.040315250120718</v>
       </c>
     </row>
     <row r="6">
@@ -655,31 +655,31 @@
         <v>0.04864900000038892</v>
       </c>
       <c r="D6" t="n">
-        <v>2935903822.5841</v>
+        <v>2934011399.472625</v>
       </c>
       <c r="E6" t="n">
-        <v>1074363717.030694</v>
+        <v>1074122075.857948</v>
       </c>
       <c r="F6" t="n">
-        <v>0.7806478376987742</v>
+        <v>0.7797390496720809</v>
       </c>
       <c r="G6" t="n">
-        <v>3416740822.5841</v>
+        <v>3414848399.472625</v>
       </c>
       <c r="H6" t="n">
-        <v>2021943485.126693</v>
+        <v>2021701843.953948</v>
       </c>
       <c r="I6" t="n">
-        <v>2.532048722576986</v>
+        <v>2.531139934550293</v>
       </c>
       <c r="J6" t="n">
-        <v>3113777187.750864</v>
+        <v>3076272471.753109</v>
       </c>
       <c r="K6" t="n">
-        <v>1139919251.494672</v>
+        <v>1139677610.321926</v>
       </c>
       <c r="L6" t="n">
-        <v>0.9414476396379265</v>
+        <v>0.9314377202680284</v>
       </c>
     </row>
     <row r="7">
@@ -693,31 +693,31 @@
         <v>0.04864900000021298</v>
       </c>
       <c r="D7" t="n">
-        <v>5705927679.578238</v>
+        <v>5630294028.144297</v>
       </c>
       <c r="E7" t="n">
-        <v>2093646234.352551</v>
+        <v>2093126971.198102</v>
       </c>
       <c r="F7" t="n">
-        <v>0.7109953314182129</v>
+        <v>0.7008739979828794</v>
       </c>
       <c r="G7" t="n">
-        <v>6610908679.578238</v>
+        <v>6535275028.144297</v>
       </c>
       <c r="H7" t="n">
-        <v>3964641970.544552</v>
+        <v>3964122707.390102</v>
       </c>
       <c r="I7" t="n">
-        <v>2.440674418878984</v>
+        <v>2.43055308544365</v>
       </c>
       <c r="J7" t="n">
-        <v>6061674413.085127</v>
+        <v>5845921493.323433</v>
       </c>
       <c r="K7" t="n">
-        <v>2224757076.981087</v>
+        <v>2224237813.826637</v>
       </c>
       <c r="L7" t="n">
-        <v>0.8717948945087223</v>
+        <v>0.8437690196521511</v>
       </c>
     </row>
     <row r="8">
@@ -731,31 +731,31 @@
         <v>0.04864900000013639</v>
       </c>
       <c r="D8" t="n">
-        <v>8377941467.746169</v>
+        <v>8213990008.872227</v>
       </c>
       <c r="E8" t="n">
-        <v>3110748851.091806</v>
+        <v>3109943213.516358</v>
       </c>
       <c r="F8" t="n">
-        <v>0.6781497591552087</v>
+        <v>0.663710703172148</v>
       </c>
       <c r="G8" t="n">
-        <v>9766021467.746168</v>
+        <v>9602070008.872227</v>
       </c>
       <c r="H8" t="n">
-        <v>5904804441.763807</v>
+        <v>5903998804.188358</v>
       </c>
       <c r="I8" t="n">
-        <v>2.403142008983776</v>
+        <v>2.388702953000714</v>
       </c>
       <c r="J8" t="n">
-        <v>8911561563.243597</v>
+        <v>8489006559.496712</v>
       </c>
       <c r="K8" t="n">
-        <v>3307415455.581211</v>
+        <v>3306609818.005763</v>
       </c>
       <c r="L8" t="n">
-        <v>0.8389495617402642</v>
+        <v>0.8024808016204954</v>
       </c>
     </row>
   </sheetData>
@@ -827,7 +827,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>6905703.521681963</v>
+        <v>31129413.79666132</v>
       </c>
     </row>
     <row r="4">
@@ -845,7 +845,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>5190165.43845242</v>
+        <v>2433142.683120457</v>
       </c>
     </row>
     <row r="5">
@@ -881,7 +881,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2929474.370415252</v>
+        <v>3704044.467577877</v>
       </c>
     </row>
     <row r="7">
@@ -935,7 +935,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6905703.521681963</v>
+        <v>31129413.79666132</v>
       </c>
     </row>
     <row r="10">
@@ -953,7 +953,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5190165.43845242</v>
+        <v>2433142.683120457</v>
       </c>
     </row>
     <row r="11">
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2929474.370415252</v>
+        <v>3704044.467577877</v>
       </c>
     </row>
     <row r="13">
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>24693040.16319393</v>
+        <v>66863779.66647149</v>
       </c>
     </row>
     <row r="15">
@@ -1043,7 +1043,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>5190165.43845242</v>
+        <v>2433142.683120457</v>
       </c>
     </row>
     <row r="16">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2929474.370415252</v>
+        <v>3704044.467577877</v>
       </c>
     </row>
     <row r="18">
@@ -1115,7 +1115,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>17264258.68303682</v>
+        <v>53942981.38183893</v>
       </c>
     </row>
     <row r="20">
@@ -1133,7 +1133,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>12975413.59512098</v>
+        <v>4216300.758467122</v>
       </c>
     </row>
     <row r="21">
@@ -1169,7 +1169,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>7323686.056924343</v>
+        <v>6418598.372623881</v>
       </c>
     </row>
     <row r="23">
@@ -1223,7 +1223,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>17264258.68303682</v>
+        <v>53942981.38183893</v>
       </c>
     </row>
     <row r="26">
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>12975413.59512098</v>
+        <v>4216300.758467122</v>
       </c>
     </row>
     <row r="27">
@@ -1277,7 +1277,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>7323686.056924343</v>
+        <v>6418598.372623881</v>
       </c>
     </row>
     <row r="29">
@@ -1313,7 +1313,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>61732599.97471839</v>
+        <v>115865709.6862738</v>
       </c>
     </row>
     <row r="31">
@@ -1331,7 +1331,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>12975413.59512098</v>
+        <v>4216300.758467122</v>
       </c>
     </row>
     <row r="32">
@@ -1367,7 +1367,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>7323686.056924343</v>
+        <v>6418598.372623881</v>
       </c>
     </row>
     <row r="34">
@@ -1403,7 +1403,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>34528517.36607379</v>
+        <v>81762270.52741547</v>
       </c>
     </row>
     <row r="36">
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>25950827.19024212</v>
+        <v>6390716.908998997</v>
       </c>
     </row>
     <row r="37">
@@ -1457,7 +1457,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>14647372.11384872</v>
+        <v>9728775.887162708</v>
       </c>
     </row>
     <row r="39">
@@ -1511,7 +1511,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>34528517.36607379</v>
+        <v>81762270.52741547</v>
       </c>
     </row>
     <row r="42">
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>25950827.19024212</v>
+        <v>6390716.908998997</v>
       </c>
     </row>
     <row r="43">
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14647372.11384872</v>
+        <v>9728775.887162708</v>
       </c>
     </row>
     <row r="45">
@@ -1601,7 +1601,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>123465199.9494373</v>
+        <v>175619575.6619699</v>
       </c>
     </row>
     <row r="47">
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>25950827.19024212</v>
+        <v>6390716.908998997</v>
       </c>
     </row>
     <row r="48">
@@ -1655,7 +1655,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>14647372.11384872</v>
+        <v>9728775.887162708</v>
       </c>
     </row>
     <row r="50">
@@ -1691,7 +1691,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>51792776.51137318</v>
+        <v>104281603.6159021</v>
       </c>
     </row>
     <row r="52">
@@ -1709,7 +1709,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>38926240.70971496</v>
+        <v>8150876.912796725</v>
       </c>
     </row>
     <row r="53">
@@ -1745,7 +1745,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>21971070.6891378</v>
+        <v>12408323.36948821</v>
       </c>
     </row>
     <row r="55">
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>51792776.51137318</v>
+        <v>104281603.6159021</v>
       </c>
     </row>
     <row r="58">
@@ -1817,7 +1817,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>38926240.70971496</v>
+        <v>8150876.912796725</v>
       </c>
     </row>
     <row r="59">
@@ -1853,7 +1853,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>21971070.6891378</v>
+        <v>12408323.36948821</v>
       </c>
     </row>
     <row r="61">
@@ -1889,7 +1889,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>185197801.5770889</v>
+        <v>223989510.788276</v>
       </c>
     </row>
     <row r="63">
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>38926240.70971496</v>
+        <v>8150876.912796725</v>
       </c>
     </row>
     <row r="64">
@@ -1943,7 +1943,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>21971070.6891378</v>
+        <v>12408323.36948821</v>
       </c>
     </row>
     <row r="66">
@@ -1979,7 +1979,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>69057034.7321621</v>
+        <v>123928427.9539241</v>
       </c>
     </row>
     <row r="68">
@@ -1997,7 +1997,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>51901654.3805984</v>
+        <v>9686515.490860688</v>
       </c>
     </row>
     <row r="69">
@@ -2033,7 +2033,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>29294744.22746908</v>
+        <v>14746066.78397044</v>
       </c>
     </row>
     <row r="71">
@@ -2087,7 +2087,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>69057034.7321621</v>
+        <v>123928427.9539241</v>
       </c>
     </row>
     <row r="74">
@@ -2105,7 +2105,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>51901654.3805984</v>
+        <v>9686515.490860688</v>
       </c>
     </row>
     <row r="75">
@@ -2141,7 +2141,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>29294744.22746908</v>
+        <v>14746066.78397044</v>
       </c>
     </row>
     <row r="77">
@@ -2177,7 +2177,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>246930399.8989262</v>
+        <v>266189500.2344076</v>
       </c>
     </row>
     <row r="79">
@@ -2195,7 +2195,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>51901654.3805984</v>
+        <v>9686515.490860688</v>
       </c>
     </row>
     <row r="80">
@@ -2231,7 +2231,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>29294744.22746908</v>
+        <v>14746066.78397044</v>
       </c>
     </row>
     <row r="82">
@@ -2267,7 +2267,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>138114070.6963407</v>
+        <v>187840372.3167065</v>
       </c>
     </row>
     <row r="84">
@@ -2285,7 +2285,7 @@
         </is>
       </c>
       <c r="D84" t="n">
-        <v>103803308.5587272</v>
+        <v>14682011.98407468</v>
       </c>
     </row>
     <row r="85">
@@ -2321,7 +2321,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>58589521.83542726</v>
+        <v>22350865.35577297</v>
       </c>
     </row>
     <row r="87">
@@ -2375,7 +2375,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>138114070.6963407</v>
+        <v>187840372.3167065</v>
       </c>
     </row>
     <row r="90">
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>103803308.5587272</v>
+        <v>14682011.98407468</v>
       </c>
     </row>
     <row r="91">
@@ -2429,7 +2429,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>58589521.83542726</v>
+        <v>22350865.35577297</v>
       </c>
     </row>
     <row r="93">
@@ -2465,7 +2465,7 @@
         </is>
       </c>
       <c r="D94" t="n">
-        <v>493860804.2032298</v>
+        <v>403467837.4958431</v>
       </c>
     </row>
     <row r="95">
@@ -2483,7 +2483,7 @@
         </is>
       </c>
       <c r="D95" t="n">
-        <v>103803308.5587272</v>
+        <v>14682011.98407468</v>
       </c>
     </row>
     <row r="96">
@@ -2519,7 +2519,7 @@
         </is>
       </c>
       <c r="D97" t="n">
-        <v>58589521.83542726</v>
+        <v>22350865.35577297</v>
       </c>
     </row>
     <row r="98">
@@ -2555,7 +2555,7 @@
         </is>
       </c>
       <c r="D99" t="n">
-        <v>207171104.1953748</v>
+        <v>239576211.7763744</v>
       </c>
     </row>
     <row r="100">
@@ -2573,7 +2573,7 @@
         </is>
       </c>
       <c r="D100" t="n">
-        <v>155704963.1402081</v>
+        <v>18725797.82477073</v>
       </c>
     </row>
     <row r="101">
@@ -2609,7 +2609,7 @@
         </is>
       </c>
       <c r="D102" t="n">
-        <v>87884232.67897314</v>
+        <v>28506831.53946798</v>
       </c>
     </row>
     <row r="103">
@@ -2663,7 +2663,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>207171104.1953748</v>
+        <v>239576211.7763744</v>
       </c>
     </row>
     <row r="106">
@@ -2681,7 +2681,7 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>155704963.1402081</v>
+        <v>18725797.82477073</v>
       </c>
     </row>
     <row r="107">
@@ -2717,7 +2717,7 @@
         </is>
       </c>
       <c r="D108" t="n">
-        <v>87884232.67897314</v>
+        <v>28506831.53946798</v>
       </c>
     </row>
     <row r="109">
@@ -2753,7 +2753,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>740791199.6928046</v>
+        <v>514592762.4008596</v>
       </c>
     </row>
     <row r="111">
@@ -2771,7 +2771,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>155704963.1402081</v>
+        <v>18725797.82477073</v>
       </c>
     </row>
     <row r="112">
@@ -2807,7 +2807,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>87884232.67897314</v>
+        <v>28506831.53946798</v>
       </c>
     </row>
   </sheetData>
@@ -2971,10 +2971,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4.218293265186338</v>
+        <v>2.389882513439421</v>
       </c>
       <c r="E7" t="n">
-        <v>33746.3461214907</v>
+        <v>19119.06010751537</v>
       </c>
     </row>
     <row r="8">
@@ -3223,10 +3223,10 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>4.218293265186338</v>
+        <v>2.389882513439421</v>
       </c>
       <c r="E19" t="n">
-        <v>33746.3461214907</v>
+        <v>19119.06010751537</v>
       </c>
     </row>
     <row r="20">
@@ -3496,10 +3496,10 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>4.218293265186338</v>
+        <v>2.389882513439421</v>
       </c>
       <c r="E32" t="n">
-        <v>33746.3461214907</v>
+        <v>19119.06010751537</v>
       </c>
     </row>
     <row r="33">
@@ -3748,10 +3748,10 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>10.54573316214491</v>
+        <v>4.538732188570339</v>
       </c>
       <c r="E44" t="n">
-        <v>84365.86529715928</v>
+        <v>36309.85750856272</v>
       </c>
     </row>
     <row r="45">
@@ -4000,10 +4000,10 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>10.54573316214491</v>
+        <v>4.538732188570339</v>
       </c>
       <c r="E56" t="n">
-        <v>84365.86529715928</v>
+        <v>36309.85750856272</v>
       </c>
     </row>
     <row r="57">
@@ -4273,10 +4273,10 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>10.54573316214491</v>
+        <v>4.538732188570339</v>
       </c>
       <c r="E69" t="n">
-        <v>84365.86529715928</v>
+        <v>36309.85750856272</v>
       </c>
     </row>
     <row r="70">
@@ -4525,10 +4525,10 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>21.09146632428995</v>
+        <v>7.373192193170913</v>
       </c>
       <c r="E81" t="n">
-        <v>168731.7305943196</v>
+        <v>58985.5375453673</v>
       </c>
     </row>
     <row r="82">
@@ -4777,10 +4777,10 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>21.09146632428995</v>
+        <v>7.373192193170913</v>
       </c>
       <c r="E93" t="n">
-        <v>168731.7305943196</v>
+        <v>58985.5375453673</v>
       </c>
     </row>
     <row r="94">
@@ -5050,10 +5050,10 @@
         </is>
       </c>
       <c r="D106" t="n">
-        <v>21.09146632428995</v>
+        <v>7.373192193170913</v>
       </c>
       <c r="E106" t="n">
-        <v>168731.7305943196</v>
+        <v>58985.5375453673</v>
       </c>
     </row>
     <row r="107">
@@ -5302,10 +5302,10 @@
         </is>
       </c>
       <c r="D118" t="n">
-        <v>31.63719942495204</v>
+        <v>9.793082999987984</v>
       </c>
       <c r="E118" t="n">
-        <v>253097.5953996163</v>
+        <v>78344.66399990387</v>
       </c>
     </row>
     <row r="119">
@@ -5554,10 +5554,10 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>31.63719942495204</v>
+        <v>9.793082999987984</v>
       </c>
       <c r="E130" t="n">
-        <v>253097.5953996163</v>
+        <v>78344.66399990387</v>
       </c>
     </row>
     <row r="131">
@@ -5827,10 +5827,10 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>31.63719942495204</v>
+        <v>9.793082999987984</v>
       </c>
       <c r="E143" t="n">
-        <v>253097.5953996163</v>
+        <v>78344.66399990387</v>
       </c>
     </row>
     <row r="144">
@@ -6079,10 +6079,10 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>42.18293264867269</v>
+        <v>11.97778605541476</v>
       </c>
       <c r="E155" t="n">
-        <v>337463.4611893815</v>
+        <v>95822.28844331812</v>
       </c>
     </row>
     <row r="156">
@@ -6331,10 +6331,10 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>42.18293264867269</v>
+        <v>11.97778605541476</v>
       </c>
       <c r="E167" t="n">
-        <v>337463.4611893815</v>
+        <v>95822.28844331812</v>
       </c>
     </row>
     <row r="168">
@@ -6604,10 +6604,10 @@
         </is>
       </c>
       <c r="D180" t="n">
-        <v>42.18293264867269</v>
+        <v>11.97778605541476</v>
       </c>
       <c r="E180" t="n">
-        <v>337463.4611893815</v>
+        <v>95822.28844331812</v>
       </c>
     </row>
     <row r="181">
@@ -6856,10 +6856,10 @@
         </is>
       </c>
       <c r="D192" t="n">
-        <v>84.36586513278876</v>
+        <v>19.45797082653878</v>
       </c>
       <c r="E192" t="n">
-        <v>674926.92106231</v>
+        <v>155663.7666123103</v>
       </c>
     </row>
     <row r="193">
@@ -7108,10 +7108,10 @@
         </is>
       </c>
       <c r="D204" t="n">
-        <v>84.36586513278876</v>
+        <v>19.45797082653878</v>
       </c>
       <c r="E204" t="n">
-        <v>674926.92106231</v>
+        <v>155663.7666123103</v>
       </c>
     </row>
     <row r="205">
@@ -7381,10 +7381,10 @@
         </is>
       </c>
       <c r="D217" t="n">
-        <v>84.36586513278876</v>
+        <v>19.45797082653878</v>
       </c>
       <c r="E217" t="n">
-        <v>674926.92106231</v>
+        <v>155663.7666123103</v>
       </c>
     </row>
     <row r="218">
@@ -7633,10 +7633,10 @@
         </is>
       </c>
       <c r="D229" t="n">
-        <v>126.5487979447281</v>
+        <v>25.84410101369209</v>
       </c>
       <c r="E229" t="n">
-        <v>1012390.383557825</v>
+        <v>206752.8081095367</v>
       </c>
     </row>
     <row r="230">
@@ -7885,10 +7885,10 @@
         </is>
       </c>
       <c r="D241" t="n">
-        <v>126.5487979447281</v>
+        <v>25.84410101369209</v>
       </c>
       <c r="E241" t="n">
-        <v>1012390.383557825</v>
+        <v>206752.8081095367</v>
       </c>
     </row>
     <row r="242">
@@ -8158,10 +8158,10 @@
         </is>
       </c>
       <c r="D254" t="n">
-        <v>126.5487979447281</v>
+        <v>25.84410101369209</v>
       </c>
       <c r="E254" t="n">
-        <v>1012390.383557825</v>
+        <v>206752.8081095367</v>
       </c>
     </row>
     <row r="255">

</xml_diff>